<commit_message>
docs: update feasibility summary for Order History epic with re-audit findings
</commit_message>
<xml_diff>
--- a/order_history/Order History - Feasibility Analysis (Consolidated).xlsx
+++ b/order_history/Order History - Feasibility Analysis (Consolidated).xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +44,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +86,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D2E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -109,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -138,6 +147,36 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -518,10 +557,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -554,7 +589,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-24 (revised after referenced stories + dependencies)</t>
+          <t>2026-06-24 (initial); RE-AUDITED 2026-06-25 under the built-write-path lens (a schema field existing is not enough — a working producer must write the data, else Blocked/Not-Deliverable)</t>
         </is>
       </c>
     </row>
@@ -566,7 +601,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>5-repo scan -&gt; per-requirement feasibility -&gt; adversarial verification of every gap -&gt; reconciliation with referenced stories -&gt; dependency mapping</t>
+          <t>5-repo scan -&gt; per-requirement feasibility -&gt; adversarial verification; 2026-06-25 producer re-audit traced the actual .create/.update write-path for every requirement (58 of 59 via workflow + #10 by analogy)</t>
         </is>
       </c>
     </row>
@@ -587,50 +622,50 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  Deliverable</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>38  (data + relations exist; needs new API/UI build only)</t>
+          <t>40  (data PRODUCED by a built write-path today; only the net-new Order History read API/UI/derivation remains)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  Partial</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>19  (partly supported; field/relation/service missing or must be derived)</t>
+          <t>13  (partly produced: only some order types/paths write the field, or a real derivation/snapshot/design caveat remains — incl. early-pay #10/#13, buildable on produced primitives but spec names a salesperson-set method that is unbuilt)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blocked</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>5  (schema may exist but NO producer writes it yet — an upstream feature is unbuilt; becomes Deliverable once it ships: Booth Number, Booth Upgrade, Onsite contact, Gift-cert redemption, Salesperson schedule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Not Deliverable</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>1  (no data/source exists today — Booth Number)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Needs Clarification</t>
-        </is>
-      </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>1  (ambiguous / architectural decision)</t>
+          <t>1  (no path even in principle — Booth Type Standard/Premium/Corner taxonomy does not exist and is unplanned)</t>
         </is>
       </c>
     </row>
@@ -654,7 +689,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>21 gap items</t>
+          <t>18 gap items</t>
         </is>
       </c>
     </row>
@@ -730,7 +765,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>DEP-1 Booth Number, DEP-2 Booth Upgrade details, DEP-3 order-level Onsite Contact, DEP-4 salesperson Payment Schedule data</t>
+          <t>DEP-1 Booth Number, DEP-2 Booth Upgrade, DEP-3 Onsite contact (producer unbuilt), DEP-4 Salesperson schedule, DEP-9 Gift-cert redemption — these gate the 5 BLOCKED items (early-pay #10/#13 is Partial: buildable now, but its salesperson-set-method framing also leans on DEP-4)</t>
         </is>
       </c>
     </row>
@@ -790,7 +825,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>The 21 Partial/Not-Deliverable/Needs-Clarification items with gap + story finding</t>
+          <t>The 19 Partial / Blocked / Not-Deliverable items with gap + producer evidence (colour-coded)</t>
         </is>
       </c>
     </row>
@@ -802,7 +837,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>10 consolidated clarification questions (4 High priority)</t>
+          <t>9 clarification questions — OQ2 &amp; OQ5 resolved 2026-06-25; 7 open (3 High). OQ5 carries a wording-flag for the BA (3-value vs 2-value payment-status labels).</t>
         </is>
       </c>
     </row>
@@ -842,7 +877,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Verdict / Priority / Dependency-type colours: Orange = blocker/High/Hard; Yellow = Partial/Medium/Soft; Blue = Needs-Clarification/Architectural; Green = Deliverable/Low</t>
+          <t>Verdict colours: Green = Deliverable, Yellow = Partial, Purple = Blocked (upstream producer unbuilt), Orange = Not Deliverable, Blue = Needs Clarification (0 left).</t>
         </is>
       </c>
     </row>
@@ -875,7 +910,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Largely deliverable but not fully. The Order data, line-item typing (booth/add-on/sponsorship/fees), installment rows, coupon/gift-cert/fee snapshots, and agreement acceptance record all exist. Shortfalls cluster into a few themes; 4 hard dependencies on out-of-scope epics.</t>
+          <t>Largely deliverable, but the built-write-path re-audit (2026-06-25) is sharper than the original: of 59 atomic requirements 40 Deliverable / 13 Partial / 5 BLOCKED / 1 Not Deliverable. KEY INSIGHT: several fields whose schema columns exist are NOT produced by any working code yet because the upstream feature is unbuilt — these are BLOCKED (become deliverable once the producer ships), not Deliverable: Onsite contact (OnsiteBoothContact table written by nothing), Gift-cert line (no giftCertificateRedeem.create anywhere), Salesperson-set payment schedule (admin writes no PaymentTransaction rows), Booth Number &amp; Booth Upgrade (planned buy-flow/Epic 7 unbuilt). Early-pay (#10/#13) is PARTIAL not Blocked (independently re-verified): a 'pay next scheduled installment now' endpoint is buildable on already-produced primitives (scheduled PaymentTransaction + saved card + off-session charge + webhook + paid-in-full fields); only the spec's 'salesperson-set payment method/schedule' wording is unbuilt (→ DEP-4, BA flag). Conversely, Invoice/Payment-Status/Associated-Shows/Booth-Size IMPROVED to Deliverable once the real producers were located (the charge-success webhook DOES create Invoice + cart-flow line-item trees for booth orders). Coupon/fee/type-discriminator fields dropped to Partial because only some checkout paths populate them (tax hardcoded 0; coupon_code vs coupon_amount split across paths).</t>
         </is>
       </c>
     </row>
@@ -899,7 +934,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Data contract now known (size increase -&gt; pay price difference -&gt; select booth number -&gt; old booth released). 'Upgrade details' moved Needs-Clarification -&gt; Partial.</t>
+          <t>Data contract now known (size increase -&gt; pay price difference -&gt; select booth number -&gt; old booth released), BUT Epic 7 is UNBUILT (verified 2026-06-25 — no upgrade flow/data in any repo). 'Upgrade details' -&gt; NOT DELIVERABLE (was Partial); nothing to display until Epic 7 ships (DEP-2).</t>
         </is>
       </c>
     </row>
@@ -935,7 +970,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Stories place onsite contact AT THE ORDER LEVEL, but schema keys (company_id, show_id) -&gt; confirmed order-linkage gap (DEP-3). Display-only for this epic.</t>
+          <t>RESOLVED 2026-06-25: per project decision we follow the DB schema (contact keyed company_id + show_id) and show ONE contact PER SHOW; the other epics' order-level framing is out of scope and disregarded. Onsite-contact display is now Deliverable; DEP-3 closed.</t>
         </is>
       </c>
     </row>
@@ -947,7 +982,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Source identified (Social Tables id chosen at selection/upgrade) but NOT persisted -&gt; remains the only Not-Deliverable item (DEP-1).</t>
+          <t>Source identified (Social Tables id chosen at selection/upgrade) but NOT persisted -&gt; Not-Deliverable (one of two, with Booth Upgrade details) (DEP-1).</t>
         </is>
       </c>
     </row>
@@ -975,7 +1010,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>A. Centralized billing service  B. Booth Number  C. Booth Size/Type (snapshot risk)  D. Booth Upgrade details  E. Per-installment Overdue  F. Order payment-status derivation  G. Order-&gt;Show link (shows/city/dates)  H. Invoice PDF  I. Pay-early endpoint  J. Payment schedule display  K. Onsite contact</t>
+          <t>A. Centralized billing (Total Amount = produced snapshot; wording Q)  B. Booth Number (BLOCKED)  C. Booth Size=Deliverable / Booth Type=Not-Deliverable  D. Booth Upgrade (BLOCKED)  E. Per-installment Overdue (Partial — not a produced status)  G. Order→Show link (Partial — derived join)  I. Early-pay (Partial — buildable on produced primitives; salesperson-set wording → DEP-4)  J. Salesperson schedule (BLOCKED)  K. Onsite contact (BLOCKED)  L. Line-item type discriminator (Partial — only cart path writes cart_item_type)  M. Coupon/fee coverage (Partial — partial producers, tax=0)  N. Gift-cert redemption (BLOCKED — no producer)</t>
         </is>
       </c>
     </row>
@@ -1193,9 +1228,9 @@
           <t>Total Amount must come from the 'centralized billing service'.</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>NeedsClarification</t>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -1205,7 +1240,9 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>No 'centralized billing service' module exists in any of the 5 repos (grep for BillingService/centralized = no hits). Order.total is a frozen SNAPSHOT computed by admin/exhibitor CartPricingService at checkout; external-api-service has zero total/subtotal/saving computation code and only persists/charges snapshots. If 'centralized billing service' means an authoritative external/separate service that must re-supply or validate the total at read time, that service does not exist and is out-of-repo/unprovided.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Producer CONFIRMED built — Order.total is frozen at checkout by CartPricingService.recalculate() (exhibitor cart-pricing.service.ts:82) via 3 real order.create paths (cart.service.ts:1221, payments.service.ts:196, admin checkout.service.ts:246). The 'centralized billing service' IS this in-process pricing engine (not a separate microservice). Data is produced today → display the snapshot. Only residual is a BA wording question (frozen snapshot vs live recompute) → moved NeedsClarification→Partial.
+— prior note —
+No 'centralized billing service' module exists in any of the 5 repos (grep for BillingService/centralized = no hits). Order.total is a frozen SNAPSHOT computed by admin/exhibitor CartPricingService at checkout; external-api-service has zero total/subtotal/saving computation code and only persists/charges snapshots. If 'centralized billing service' means an authoritative external/separate service that must re-supply or validate the total at read time, that service does not exist and is out-of-repo/unprovided.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -1238,9 +1275,9 @@
           <t>Column: Payment Status — order-level status derived from associated payment plan / installment statuses (Paid in Full / Partially Paid / Unpaid).</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -1250,7 +1287,9 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>OrderStatus enum (schema:418) has only pending|partially_paid|completed|failed|refunded|canceled — NO literal 'unpaid' or 'paid in full'. Raw inputs exist (Order.paid_amount, paid_in_full_at, partially_paid; PaymentTransaction.status per installment) but the Paid in Full / Partially Paid / Unpaid mapping must be DERIVED in a new service (compare paid_amount vs total, roll up PaymentTransaction rows). No read-side derivation logic exists in exhibitor-backend-api.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Producer CONFIRMED — Order.status/paid_amount/paid_in_full_at written at checkout (status=pending) then by the external-api webhook on each succeeded installment (webhook.service.ts:2098 via computeNewOrderStatus → completed/partially_paid); PaymentTransaction rows produced by the split loop (payments.service.ts:261). All Paid-in-Full/Partially-Paid/Unpaid inputs are produced by working code; only the read derivation remains → Deliverable.
+— prior note —
+OrderStatus enum (schema:418) has only pending|partially_paid|completed|failed|refunded|canceled — NO literal 'unpaid' or 'paid in full'. Raw inputs exist (Order.paid_amount, paid_in_full_at, partially_paid; PaymentTransaction.status per installment) but the Paid in Full / Partially Paid / Unpaid mapping must be DERIVED in a new service (compare paid_amount vs total, roll up PaymentTransaction rows). No read-side derivation logic exists in exhibitor-backend-api.</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr"/>
@@ -1320,9 +1359,9 @@
           <t>Column: Associated Shows (multi-city / multi-show) per order.</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -1332,7 +1371,9 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Order has NO direct show_id (verified at schema.prisma:1532-1596 — no show_id/show relation). Associated Shows is derivable ONLY via OrderItem.show_product_id (schema:1931) -&gt; ShowProduct.show_id (schema:2627) -&gt; Shows. Grouping/join logic must be built. Subscription/ppl_addon order_types have no show_product_id and therefore no associated shows.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Producer CONFIRMED — OrderItem.show_product_id written at checkout (cart.helpers.ts:55; admin checkout.service.ts:266/275). Orders are company-scoped and legitimately multi-show; Associated Shows = OrderItem.show_product_id→ShowProduct→Shows, a pure read join over produced data → Deliverable. (Non-show order types simply have no shows — expected.)
+— prior note —
+Order has NO direct show_id (verified at schema.prisma:1532-1596 — no show_id/show relation). Associated Shows is derivable ONLY via OrderItem.show_product_id (schema:1931) -&gt; ShowProduct.show_id (schema:2627) -&gt; Shows. Grouping/join logic must be built. Subscription/ppl_addon order_types have no show_product_id and therefore no associated shows.</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr"/>
@@ -1402,9 +1443,9 @@
           <t>Action: Invoice (download/view invoice PDF).</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1414,7 +1455,9 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Invoice/InvoiceLineItem data models exist (schema:1953/1987) but Invoice has NO file_url/PDF field and no stored invoice document. A working pdfkit renderer exists but is PPL-specific (exhibitor-backend-api/src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf + S3). A product/booth order invoice PDF renderer must be generalized/built; no invoice-PDF route exists for order-history.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Producer CONFIRMED (first auditor missed it) — the charge-success webhook creates Invoice (webhook.service.ts:2048) + InvoiceLineItems for EVERY non-subscription order on payment success; cart-flow/booth orders materialize as a tree (materializeOrderItemsToCartInvoiceLines, :2072). Invoice DATA is produced for booth/product orders. Remaining work = generalize the today-PPL-only pdfkit renderer + add a download route (net-new read layer). Caveat: invoice exists only AFTER a successful installment (one per installment in split mode) → Deliverable.
+— prior note —
+Invoice/InvoiceLineItem data models exist (schema:1953/1987) but Invoice has NO file_url/PDF field and no stored invoice document. A working pdfkit renderer exists but is PPL-specific (exhibitor-backend-api/src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf + S3). A product/booth order invoice PDF renderer must be generalized/built; no invoice-PDF route exists for order-history.</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr"/>
@@ -1455,7 +1498,11 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Charge primitives exist (external-api-service stripe.service.createPaymentIntent + saved PaymentMethod brand/last4 + PaymentTransaction.source=manual_retry) but NO endpoint to pay an existing order's outstanding/scheduled installment EARLY. exhibitor-backend-api payments module exposes only POST /payments/checkout (creates a NEW order); there is no 'pay scheduled installment ahead of schedule' route. Depends on external stories Payment Schedule Visibility and Credit Card Payment Workflow (unprovided). The 'NOT Paid in Full' gating reuses the same payment-status derivation gap (no unpaid/paid-in-full enum literal).</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (INDEPENDENT single-item audit): moved Blocked→Partial. The early-pay action rests on ALREADY-PRODUCED primitives — scheduled PaymentTransaction rows carry a saved card (stripe_payment_method_id) + due_date, produced by exhibitor split checkout (payments.service.ts:261-284); the off-session charge primitive (the same one the daily cron calls), webhook reconciliation, and paid-in-full gating (Order.paid_amount/paid_in_full_at, schema:1565-66) all exist. A net-new 'pay next scheduled installment now' endpoint is buildable on these TODAY → Partial. ⚑ BA FLAG: the spec's 'salesperson-set payment method' does NOT exist (the card is the exhibitor's own) and the schedule is system-generated (fixed 30-day cadence via INSTALLMENT_INTERVAL_DAYS), not salesperson-authored — that salesperson-origination model is the separate Blocked item #56/DEP-4. On the literal salesperson-driven reading this tips to Blocked/NeedsClarification; on the as-built exhibitor self-service reading it is Partial.
+— earlier re-audit note —
+⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED — twin of #13 (the re-audit agent hit a tool error here; verdict assigned by analogy with adversarially-confirmed #13). Same blockers: no salesperson-set payment method/schedule producer + no pay-existing-order endpoint.
+— prior note —
+Charge primitives exist (external-api-service stripe.service.createPaymentIntent + saved PaymentMethod brand/last4 + PaymentTransaction.source=manual_retry) but NO endpoint to pay an existing order's outstanding/scheduled installment EARLY. exhibitor-backend-api payments module exposes only POST /payments/checkout (creates a NEW order); there is no 'pay scheduled installment ahead of schedule' route. Depends on external stories Payment Schedule Visibility and Credit Card Payment Workflow (unprovided). The 'NOT Paid in Full' gating reuses the same payment-status derivation gap (no unpaid/paid-in-full enum literal).</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1500,10 +1547,16 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>PaymentTransactionStatus enum (admin-backend-api/prisma/schema.prisma:488) has NO 'overdue' value (scheduled|processing|succeeded|failed|canceled|refunded). 'Overdue' is not a stored state. Two paths: (a) DERIVE at read time = status in (scheduled,failed) AND due_date &lt; now() - no migration, computed in exhibitor-backend-api read service; OR (b) add an 'overdue' enum value + an overdue-marking cron. background-worker-service has the cron home (cart-maintenance.expireCarts is the template) and reads @@index([status,due_date]) already, but enum/migration must be added in admin-backend-api (migration source of truth). If only derive-at-read is needed, this is Deliverable; the Partial reflects that no stored Overdue state exists today.</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr"/>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: 'Overdue' is NOT a produced status — no overdue enum and no write-path sets one; a past-due installment stays status=scheduled and the daily cron will actually attempt to charge it (scheduled→processing→succeeded/failed), so overdue is a transient/derived state with real lifecycle caveats, not a stored value. Derivable but caveated → Partial.
+— prior note —
+DELIVERABLE (re-audit 2026-06-25, adversarially confirmed, high confidence): all inputs exist and are actively produced — each installment is a real PaymentTransaction row with a populated due_date + status, written by checkout, the daily charge cron, and Stripe webhooks. 'Overdue' = status NOT IN (succeeded,refunded,canceled) AND due_date &lt; now() — a mechanical read-time derivation over the existing @@index([status,due_date]). The missing 'overdue' enum literal is a presentation convenience, not a data gap; no upstream feature is needed. (Was Partial.)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Re-audited Partial→Deliverable. Opposite of the Booth-Upgrade failure mode: data is fully present and live. Inputs: PaymentTransaction.due_date/status (admin schema:2055/2060) + @@index([status,due_date]):2077; rows created in payments.service.ts (split loop) + checkout.service.ts; consumed by worker payment-charge cron.</t>
+        </is>
+      </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Enum at schema.prisma:488-497 lacks 'overdue'; grep 'overdue' across worker src finds only lead-distribution doc comments; PaymentTransaction.due_date (schema:2060) + @@index([status,due_date]) (2077) provide the derivation inputs.</t>
@@ -1529,9 +1582,9 @@
           <t>Invoice action: download/view the order Invoice as a PDF.</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1541,7 +1594,9 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>No order-invoice PDF generator and no stored invoice file. Invoice model has NO file_url/PDF field (exhibitor-backend-api prisma/schema.prisma:1953; only file_url at line 348 is the Agreement TEMPLATE). A working pdfkit renderer exists but is PPL-specific (src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf, line 985/753) and would need generalization to product/booth orders from Invoice + InvoiceLineItem. No invoice-PDF route or service for orders exists in any repo (external-api-service and background-worker-service both lack PDF tooling).</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Producer CONFIRMED — same as #9: charge-success webhook creates Invoice (webhook.service.ts:2048) + cart-flow line-item tree (:2072) for booth/product orders. Data produced; remaining = generalize PPL-only renderer + add route. → Deliverable (caveat: invoice produced post-payment, one per installment).
+— prior note —
+No order-invoice PDF generator and no stored invoice file. Invoice model has NO file_url/PDF field (exhibitor-backend-api prisma/schema.prisma:1953; only file_url at line 348 is the Agreement TEMPLATE). A working pdfkit renderer exists but is PPL-specific (src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf, line 985/753) and would need generalization to product/booth orders from Invoice + InvoiceLineItem. No invoice-PDF route or service for orders exists in any repo (external-api-service and background-worker-service both lack PDF tooling).</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
@@ -1582,7 +1637,11 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>No endpoint to pay an EXISTING order's outstanding/future scheduled installment. exhibitor-backend-api payments controller exposes ONLY POST /payments/checkout (src/payments/controllers/payments.controller.ts:50) — a cart-&gt;order creation flow, not pay-an-existing-order. external-api-service has charge primitives (stripe.service.createPaymentIntent, saved PaymentMethod brand/last4, PaymentTransaction.source=manual_retry) but NO dedicated early-pay/pay-now controller route. A new 'pay order' endpoint must be built that selects scheduled PaymentTransaction rows (status=scheduled, future due_date), charges them off-schedule via the salesperson-set stripe_payment_method_id + a card, and reconciles paid_amount via the existing external-api webhook. Depends on external stories Payment Schedule Visibility + Credit Card Payment Workflow which define the redirect/payment-summary UX and which card/method is authoritative.</t>
+          <t>⟳ RE-AUDIT 2026-06-25: revised Blocked→Partial to match its independently-verified twin #10. The batch audit's Blocked call over-weighted the 'salesperson-set method/schedule' wording; the early-pay capability itself is buildable on produced primitives (scheduled PaymentTransaction + saved card + off-session charge + webhook + paid-in-full fields). The pure salesperson-origination dependency remains Blocked as #56 (DEP-4). ⚑ BA flag retained on the 'salesperson-set payment method' wording.
+— earlier re-audit note —
+⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED (producer unbuilt): both premises depend on unbuilt upstream features. (1) No salesperson-set schedule/method — every PaymentTransaction producer generates a SYSTEM equal-split with fixed 30-day cadence (payments.service.ts:261/276; INSTALLMENT_INTERVAL_DAYS=30); admin/staff checkout writes NO PaymentTransaction rows. (2) No early-pay endpoint — only POST /payments/checkout exists. Becomes Deliverable once salesperson scheduling (DEP-4) + a pay-existing-order endpoint ship.
+— prior note —
+No endpoint to pay an EXISTING order's outstanding/future scheduled installment. exhibitor-backend-api payments controller exposes ONLY POST /payments/checkout (src/payments/controllers/payments.controller.ts:50) — a cart-&gt;order creation flow, not pay-an-existing-order. external-api-service has charge primitives (stripe.service.createPaymentIntent, saved PaymentMethod brand/last4, PaymentTransaction.source=manual_retry) but NO dedicated early-pay/pay-now controller route. A new 'pay order' endpoint must be built that selects scheduled PaymentTransaction rows (status=scheduled, future due_date), charges them off-schedule via the salesperson-set stripe_payment_method_id + a card, and reconciles paid_amount via the existing external-api webhook. Depends on external stories Payment Schedule Visibility + Credit Card Payment Workflow which define the redirect/payment-summary UX and which card/method is authoritative.</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -2059,9 +2118,9 @@
           <t>Booth Number</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>NotDeliverable</t>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -2071,7 +2130,9 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>No booth_number / boothNumber field exists anywhere in schema or code (grep over both prisma schemas and src returned no matches). OrderItem has NO metadata column (only description VarChar(255)); the free-form JsonB 'metadata' (booth size/show title) exists ONLY on CartItem, and is NOT carried onto OrderItem at checkout. So there is no stored or derivable source for a per-order assigned Booth Number. Requires a new column (migration owned by admin-backend-api; exhibitor repo uses db push) and a write path to populate it, or an external assignment source. SOURCE now identified (Social Tables booth identifier selected at booth selection/upgrade), but it is still NOT persisted on Order/OrderItem — a column + write path from the booth-selection flow is required.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Reclassified NotDeliverable→Blocked under the new taxonomy: Booth Number has no column and NO producer today (0 hits across 5 repos; no Social Tables integration), but its producer is a PLANNED upstream feature — the Social Tables booth id chosen in the booth-selection/upgrade buy-flow (DEP-1). Planned-but-unbuilt = Blocked (becomes deliverable once the buy-flow persists it), not NotDeliverable.
+— prior note —
+No booth_number / boothNumber field exists anywhere in schema or code (grep over both prisma schemas and src returned no matches). OrderItem has NO metadata column (only description VarChar(255)); the free-form JsonB 'metadata' (booth size/show title) exists ONLY on CartItem, and is NOT carried onto OrderItem at checkout. So there is no stored or derivable source for a per-order assigned Booth Number. Requires a new column (migration owned by admin-backend-api; exhibitor repo uses db push) and a write path to populate it, or an external assignment source. SOURCE now identified (Social Tables booth identifier selected at booth selection/upgrade), but it is still NOT persisted on Order/OrderItem — a column + write path from the booth-selection flow is required.</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -2227,9 +2288,9 @@
           <t>Header: Payment Status</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -2239,7 +2300,9 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>OrderStatus enum has pending|partially_paid|completed|failed|refunded|canceled but NO literal 'unpaid'/'overdue' value. The required Paid-in-Full / Partially Paid / Unpaid (and Overdue reflected as not-fully-paid) must be DERIVED in code from Order.paid_amount vs Order.total + Order.paid_in_full_at and per-installment PaymentTransaction.status/due_date (overdue = status in scheduled/failed AND due_date&lt;now). Raw data is fully present; derivation service is unbuilt in the read repo.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Producer CONFIRMED — Order.status produced end-to-end: written pending at checkout, transitioned by the live webhook (webhook.service.ts:2098) to completed/partially_paid/failed/canceled with paid_amount/paid_in_full_at. The 3-value header status is a mechanical read derivation over produced data → Deliverable.
+— prior note —
+OrderStatus enum has pending|partially_paid|completed|failed|refunded|canceled but NO literal 'unpaid'/'overdue' value. The required Paid-in-Full / Partially Paid / Unpaid (and Overdue reflected as not-fully-paid) must be DERIVED in code from Order.paid_amount vs Order.total + Order.paid_in_full_at and per-installment PaymentTransaction.status/due_date (overdue = status in scheduled/failed AND due_date&lt;now). Raw data is fully present; derivation service is unbuilt in the read repo.</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -2268,9 +2331,9 @@
           <t>Booth Size (e.g. 10x10)</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -2280,7 +2343,9 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>No booth-size field on OrderItem; size is derivable from Product.length/width (Decimal) via OrderItem.product_id -&gt; Product, since the booth is modeled as a Product. This is a snapshot risk: OrderItem.description is the only frozen name snapshot; length/width are read live off the current Product, so if the product is later edited the displayed size may drift from purchase time. Derivation/formatting (length x width) must be built; consider snapshotting at checkout.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Producer CONFIRMED — Product.length/width written by product-management create/update (product-management.service.ts:1151-1152) and REQUIRED for Booth/Workshop-Pavilion families; OrderItem→Product link produced at checkout. Booth Size = join + format LxW, pure read derivation over produced data → Deliverable. (Minor: size read live off Product, not frozen on the line — snapshot-drift caveat.)
+— prior note —
+No booth-size field on OrderItem; size is derivable from Product.length/width (Decimal) via OrderItem.product_id -&gt; Product, since the booth is modeled as a Product. This is a snapshot risk: OrderItem.description is the only frozen name snapshot; length/width are read live off the current Product, so if the product is later edited the displayed size may drift from purchase time. Derivation/formatting (length x width) must be built; consider snapshotting at checkout.</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr"/>
@@ -2309,9 +2374,9 @@
           <t>Booth Type (Standard/Premium/Corner)</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>NotDeliverable</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -2321,10 +2386,14 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>No first-class Booth Type on the order line. ProductType hierarchy (ProductType.name/code, parent_type_id) classifies products as booth/sponsor/etc., but there is no confirmed Standard/Premium/Corner taxonomy in the schema/seed (no such ProductType codes found). Booth Type would be derived from OrderItem.product -&gt; Product.product_type_id -&gt; ProductType, but the exact Standard/Premium/Corner values are not modeled/seeded today, so the mapping is unproven. Same live-vs-snapshot drift risk as Booth Size.</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr"/>
+          <t>NOT DELIVERABLE (re-audit 2026-06-25, adversarially confirmed, high confidence): the Standard/Premium/Corner booth-type taxonomy does NOT exist anywhere — no booth_type/tier column on Product or OrderItem, and the ProductType 'Booth' hierarchy has only two leaves ('Booth' [code booth_standard] and 'Workshop Pavilion'), which are product FAMILIES, not tiers. 'booth_standard' is a false friend (its display name is just 'Booth'); zero matches for a Premium or Corner booth type; no floor-plan geometry exists to derive Corner. Same failure mode as Booth Upgrade — nothing to render until an upstream booth-type taxonomy (column/enum + admin authoring + capture on the order line) is built. (Was Partial.)</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Re-audited Partial→NotDeliverable. The tier classification produces no data; cannot build on existing data. product-type.constants.ts:19-22 = only {STANDARD:'booth_standard', WORKSHOP_PAVILION:'workshop_pavilion'}; 'premium'/'corner' have zero booth-type matches across all repos.</t>
+        </is>
+      </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
           <t>ProductType model (name VarChar(100), code unique, parent_type_id hierarchy) admin schema; no Standard/Premium/Corner codes found in schema/seed. Reached via OrderItem.product_id -&gt; Product.product_type_id -&gt; ProductType. No booth_type column on OrderItem.</t>
@@ -2350,9 +2419,9 @@
           <t>Upgrade details (if any)</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2362,12 +2431,14 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Data contract now known, but no dedicated upgrade fields in schema. Upgrade likely = a price-difference OrderItem (parent_order_item_id tree / cart_item_type) + capture of from-size/to-size + new booth number. Needs storage design + write path; no from/to-size or upgrade-delta column exists today.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Reclassified NotDeliverable→Blocked: Booth Upgrade (Epic 7) is entirely unbuilt (0 upgrade producers across 5 repos) but is a PLANNED epic with a known data contract (size↑ → price diff → new booth → old released). Planned-but-unbuilt upstream = Blocked; becomes deliverable once Epic 7 ships (DEP-2).
+— prior note —
+NOT DELIVERABLE: the Booth Upgrade feature itself (Epic 7) is NOT implemented anywhere in the codebase (verified 2026-06-25 — no upgrade flow, no price-difference/from-size/to-size/release-booth logic, no upgrade or booth_number fields in the source-of-truth schema; the only 'upgrade' code hits are PPL plan change, WebSocket protocol upgrade, a Nunify webhook flag, and a test-fixture string). With no upstream feature and no data produced, Order History has nothing to display. Blocked by DEP-2.</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>RESOLVED by Booth Upgrade story (Epic 7.1/7.2). Upgrade = pick larger size -&gt; pay PRICE DIFFERENCE (computed by 'centralized pricing service') -&gt; select new booth number -&gt; old booth released. 'Upgrade details' to render = from-size -&gt; to-size, upgrade amount, new booth number.</t>
+          <t>Booth Upgrade story (Epic 7.1/7.2) defines the intended contract (pick larger size → pay price difference → select new booth number → old booth released), but Epic 7 is out of scope AND unbuilt, so no upgrade record exists to render. Reclassified Partial → Not Deliverable on 2026-06-25.</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -2395,9 +2466,9 @@
           <t>Total Saving Made = actual price vs sales price, COMPUTED BY centralized billing service</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -2407,12 +2478,12 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>The savings VALUE exists as a frozen snapshot (Order.total_savings, schema:1571 = sum of (actual - sales) deltas captured at order creation by admin CartPricingService). But there is NO 'centralized billing service' module in any of the 5 repos: billing math is split between cart-pricing (admin-backend-api) and payment/invoice handling (external-api-service). external-api-service explicitly has zero total/saving computation code (all are upstream snapshots). If the requirement mandates a single authoritative centralized billing service to (re)compute Total Saving Made, that service does not exist; if displaying the stored Order.total_savings (with per-line backing via InvoiceLineItem.original_price vs unit_price / ShowProduct.actual_price vs sales_price) suffices, it is Deliverable.</t>
+          <t>DELIVERABLE (re-audit 2026-06-25, adversarially confirmed, medium confidence): the gap's premise that 'no centralized billing service exists' is FALSE — CartPricingService (admin + exhibitor) is the documented 'SINGLE source of truth for all cart money' and computes total_savings = Σ max(0, actual−sale)×qty, frozen onto Order.total_savings at order creation (cart.service.ts:1222). Both readings satisfied: display the stored snapshot (read-only) OR reuse the existing engine to recompute. Only caveat is inherent snapshot drift (expected for an order record). NOTE: OQ1 (read-only display vs. build a service) stays open as a scope question, but the data AND a centralized engine both already exist. (Was Partial.)</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>'Centralized billing/pricing service' is a SYSTEM-WIDE concept (also in Booth Upgrade &amp; Recommended Upsell). No such discrete service exists; pricing lives in cart-pricing (admin + exhibitor) as snapshots. For read-only Order History the snapshot on Order.total / Order.total_savings is the natural source. See DEP-7.</t>
+          <t>Re-audited Partial→Deliverable. CartPricingService:55 (admin) = centralized engine; exhibitor mirror cart-pricing.service.ts:138-139 computes per-unit saving. Order.total_savings (admin schema:1571) populated. InvoiceLineItem per-line backing is unused (no invoiceLineItem.create anywhere), but the order-level snapshot is the requirement's real data point.</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
@@ -2440,9 +2511,9 @@
           <t>Download invoice (per-order / per-payment invoice document)</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -2452,7 +2523,9 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Invoice/InvoiceLineItem data rows exist (with InvoiceItemType covering booth/addon/sponsorship/fees and original_price vs unit_price for savings), but Invoice has NO file_url/PDF storage field and there is no order/booth invoice PDF renderer. A working pdfkit renderer exists at exhibitor-backend-api src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf with S3 upload, but it is PPL-invoice-specific and would need to be generalized to product/booth orders. Missing: a generalized order-invoice PDF renderer + download endpoint (no schema change strictly required since generation can be on-demand).</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Adversarial challenge OVERTURNED Partial→Deliverable: found 3 live InvoiceLineItem producers the first auditor missed (webhook.service.ts:762 createMany, :2225 + :2414 create). Booth/cart orders get Invoice + line-item rows produced on payment success (:2048/:2072). Data produced; remaining = generalize the PPL-only PDF renderer + download route. Caveat: invoice produced post-payment, per installment (matches 'per-order/per-payment') → Deliverable.
+— prior note —
+Invoice/InvoiceLineItem data rows exist (with InvoiceItemType covering booth/addon/sponsorship/fees and original_price vs unit_price for savings), but Invoice has NO file_url/PDF storage field and there is no order/booth invoice PDF renderer. A working pdfkit renderer exists at exhibitor-backend-api src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf with S3 upload, but it is PPL-invoice-specific and would need to be generalized to product/booth orders. Missing: a generalized order-invoice PDF renderer + download endpoint (no schema change strictly required since generation can be on-demand).</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr"/>
@@ -2481,9 +2554,9 @@
           <t>Display onsite booth contact information (name/email/phone) for the order</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -2493,12 +2566,14 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>CONFIRMED gap: stories want an order-level onsite contact, but OnsiteBoothContact is keyed (company_id, show_id) with NO order linkage. Resolve multi-show (one order spanning shows -&gt; multiple per-show contacts). Display-only for this epic.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED (producer unbuilt): the OnsiteBoothContact table exists (migration 20260622120000) but ZERO code writes it — no onsiteBoothContact.create/upsert/update anywhere in 5 repos. Schema doc-comment names the producer as the unbuilt 'Exhibitor Onboarding → Onsite Booth Contacts' step (later synced to HubSpot/order). The per-show display decision stands, but there is no produced data to show until that step ships → Blocked (was Deliverable; reopens DEP-3 on producer grounds).
+— prior note —
+RESOLVED (decision 2026-06-25): show ONE onsite contact PER SHOW, sourced from OnsiteBoothContact via Order.company_id + (OrderItem.show_product_id → ShowProduct → Shows).show_id. No order-level link needed; the conflicting order-level framing from epics 16/22 is out of scope and disregarded. Shows with no contact yet render a placeholder.</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>View Onsite Booth Contact (16.1) + Onsite Contacts Management (22.4) + HubSpot Sync (22.5) explicitly place the onsite contact AT THE ORDER LEVEL. Order History only DISPLAYS it (View); Edit/HubSpot sync are separate epics (see DEP-3).</t>
+          <t>13.3 mandates displaying onsite contact and defers the contract to 'View Onsite Booth Contact' (16.1/22.4/22.5), which assumes an order-level contact. Per project decision we follow the schema instead (per-show). Edit + HubSpot sync remain epics 16/22.</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -2748,9 +2823,9 @@
           <t>OrderItem records carry a type discriminator that separates booth, add-on, and sponsorship lines so the details page can render distinct sections with qty + unit price</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -2760,7 +2835,9 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Minor: cart_item_type is nullable (CartItemType?). For cart-originated booth/add-on/sponsorship product orders (the scope of 13.3) it is populated from the cart line, but subscription/ppl_addon orders leave it null. The read service must treat null as 'not a sectioned product line', which is correct for those order types. No data-model gap for the in-scope sections.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: the booth/add-on/sponsorship discriminator is the NULLABLE OrderItem.cart_item_type, produced by only ONE of four order-creating paths — the exhibitor self-service cart checkout (cart.helpers.ts:52). Admin/staff checkout, the installment-payments path, and PPL paths leave it null, so those orders cannot be sectioned. Buildable for cart-origin product orders only → Partial.
+— prior note —
+Minor: cart_item_type is nullable (CartItemType?). For cart-originated booth/add-on/sponsorship product orders (the scope of 13.3) it is populated from the cart line, but subscription/ppl_addon orders leave it null. The read service must treat null as 'not a sectioned product line', which is correct for those order types. No data-model gap for the in-scope sections.</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr"/>
@@ -2826,9 +2903,9 @@
           <t>Discount / Coupon Code line (amount and applied code), shown when applied</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
@@ -2838,7 +2915,9 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Coupon-to-order link is a snapshot only (Order.coupon_code + Order.coupon_amount); the CouponOrders join table is commented out (schema ~1752-1768). Sufficient for displaying the applied code + discount amount; no normalized relation to the CouponCode definition for richer detail.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: on the exhibitor side neither built path produces BOTH coupon fields together — the product-cart path writes coupon_amount but never coupon_code (so 'applied code' is null when a discount applied), and the PPL/addon path writes coupon_code but hardcodes coupon_amount=0 (Phase-2 TODO). Only admin checkout writes both. Coupon line degrades on exhibitor self-serve orders → Partial.
+— prior note —
+Coupon-to-order link is a snapshot only (Order.coupon_code + Order.coupon_amount); the CouponOrders join table is commented out (schema ~1752-1768). Sufficient for displaying the applied code + discount amount; no normalized relation to the CouponCode definition for richer detail.</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr"/>
@@ -2867,9 +2946,9 @@
           <t>Gift Certificate line (applied gift-certificate amount), shown when applied</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2877,7 +2956,11 @@
           <t>exhibitor-backend-api</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED (producer unbuilt): NO giftCertificateRedeem.create/update anywhere — only admin read-reports (findMany/aggregate). GiftCertificatePurchase is also never created; only GiftCertificate definitions are written. The redemption/consumption flow that links a gift cert to an order and writes the applied amount does not exist → Blocked (new DEP-9; becomes deliverable once the redeem flow ships).</t>
+        </is>
+      </c>
       <c r="H47" s="5" t="inlineStr"/>
       <c r="I47" s="5" t="inlineStr">
         <is>
@@ -3015,9 +3098,9 @@
           <t>Conditional display of summary lines (discount/coupon/gift cert, cleaning fee, setup fee only when applicable)</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
@@ -3025,7 +3108,11 @@
           <t>exhibitor-backend-api</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: mixed producer coverage. Coupon line produced by all paths; setup/cleaning fees produced only by product-cart + admin checkout (NOT the installment-payments or PPL paths); the gift-cert line has NO producer at all (see #46). Conditional display is buildable for product-cart orders but degenerate for others → Partial.</t>
+        </is>
+      </c>
       <c r="H51" s="5" t="inlineStr"/>
       <c r="I51" s="5" t="inlineStr">
         <is>
@@ -3097,9 +3184,9 @@
           <t>Each fee/field has backing data verified</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -3107,7 +3194,11 @@
           <t>exhibitor-backend-api</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr"/>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: most fields have real producers, but two fail 'each fee/field has backing data' — TAX is hardcoded to 0 in both order producers (cart-pricing.service.ts:173, payments.service.ts:525 — Phase-2 TODO) and the gift-cert field has no producer (#46). Not every fee/field is genuinely backed by produced data → Partial.</t>
+        </is>
+      </c>
       <c r="H53" s="5" t="inlineStr"/>
       <c r="I53" s="5" t="inlineStr">
         <is>
@@ -3245,9 +3336,9 @@
           <t>Display payment schedule set by salesperson (installment dates + amounts + method)</t>
         </is>
       </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
@@ -3257,7 +3348,9 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>DISPLAY is deliverable from PaymentTransaction (installment_number, due_date, amount, status, stripe_payment_method_id). Salesperson ORIGINATION of a custom schedule is an ADMIN/salesperson-epic dependency (see DEP-4), not an Order History gap.</t>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED (producer unbuilt): this requirement is the schedule 'set by SALESPERSON'. admin-backend-api writes ZERO PaymentTransaction rows (createOrderFromCart creates none); every built installment producer is exhibitor self-service generating a SYSTEM equal-split (fixed cadence), not salesperson-authored dates/amounts/method → Blocked (DEP-4). Read-only display of the SYSTEM schedule would be deliverable, but the salesperson-origination this req names is unbuilt.
+— prior note —
+DISPLAY is deliverable from PaymentTransaction (installment_number, due_date, amount, status, stripe_payment_method_id). Salesperson ORIGINATION of a custom schedule is an ADMIN/salesperson-epic dependency (see DEP-4), not an Order History gap.</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
@@ -3393,7 +3486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3461,996 +3554,936 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>C. Booth Size / Type</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Booth/Workshop Pavilion section</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Booth Type (Standard/Premium/Corner)</t>
+        </is>
+      </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>NotDeliverable</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>NOT DELIVERABLE (re-audit 2026-06-25, adversarially confirmed, high confidence): the Standard/Premium/Corner booth-type taxonomy does NOT exist anywhere — no booth_type/tier column on Product or OrderItem, and the ProductType 'Booth' hierarchy has only two leaves ('Booth' [code booth_standard] and 'Workshop Pavilion'), which are product FAMILIES, not tiers. 'booth_standard' is a false friend (its display name is just 'Booth'); zero matches for a Premium or Corner booth type; no floor-plan geometry exists to derive Corner. Same failure mode as Booth Upgrade — nothing to render until an upstream booth-type taxonomy (column/enum + admin authoring + capture on the order line) is built. (Was Partial.)</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Re-audited Partial→NotDeliverable. The tier classification produces no data; cannot build on existing data. product-type.constants.ts:19-22 = only {STANDARD:'booth_standard', WORKSHOP_PAVILION:'workshop_pavilion'}; 'premium'/'corner' have zero booth-type matches across all repos.</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>ProductType model (name VarChar(100), code unique, parent_type_id hierarchy) admin schema; no Standard/Premium/Corner codes found in schema/seed. Reached via OrderItem.product_id -&gt; Product.product_type_id -&gt; ProductType. No booth_type column on OrderItem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>B. Booth Number (BLOCKED — DEP-1)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Booth/Workshop Pavilion section</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Booth Number</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>admin-backend-api, exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Reclassified NotDeliverable→Blocked under the new taxonomy: Booth Number has no column and NO producer today (0 hits across 5 repos; no Social Tables integration), but its producer is a PLANNED upstream feature — the Social Tables booth id chosen in the booth-selection/upgrade buy-flow (DEP-1). Planned-but-unbuilt = Blocked (becomes deliverable once the buy-flow persists it), not NotDeliverable.
+— prior note —
+No booth_number / boothNumber field exists anywhere in schema or code (grep over both prisma schemas and src returned no matches). OrderItem has NO metadata column (only description VarChar(255)); the free-form JsonB 'metadata' (booth size/show title) exists ONLY on CartItem, and is NOT carried onto OrderItem at checkout. So there is no stored or derivable source for a per-order assigned Booth Number. Requires a new column (migration owned by admin-backend-api; exhibitor repo uses db push) and a write path to populate it, or an external assignment source. SOURCE now identified (Social Tables booth identifier selected at booth selection/upgrade), but it is still NOT persisted on Order/OrderItem — a column + write path from the booth-selection flow is required.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Booth Upgrade story 7.2 step 4: 'the Exhibitor shall select a booth number'; Social Tables provides booth identifiers (Booth ID/Size/Location). So Booth Number = the Social Tables booth ID chosen at booth selection/upgrade.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>grep booth_number/boothNumber = 0 hits across admin-backend-api/prisma/schema.prisma + exhibitor-backend-api/prisma/schema.prisma + src. OrderItem model (admin schema:1919-1950) has no metadata/booth_number field; only CartItem.metadata JsonB (schema:2819) snapshots 'booth size, show title'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>D. Booth Upgrade (BLOCKED — DEP-2)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Booth/Workshop Pavilion section</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Upgrade details (if any)</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api, admin-backend-api</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Reclassified NotDeliverable→Blocked: Booth Upgrade (Epic 7) is entirely unbuilt (0 upgrade producers across 5 repos) but is a PLANNED epic with a known data contract (size↑ → price diff → new booth → old released). Planned-but-unbuilt upstream = Blocked; becomes deliverable once Epic 7 ships (DEP-2).
+— prior note —
+NOT DELIVERABLE: the Booth Upgrade feature itself (Epic 7) is NOT implemented anywhere in the codebase (verified 2026-06-25 — no upgrade flow, no price-difference/from-size/to-size/release-booth logic, no upgrade or booth_number fields in the source-of-truth schema; the only 'upgrade' code hits are PPL plan change, WebSocket protocol upgrade, a Nunify webhook flag, and a test-fixture string). With no upstream feature and no data produced, Order History has nothing to display. Blocked by DEP-2.</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Booth Upgrade story (Epic 7.1/7.2) defines the intended contract (pick larger size → pay price difference → select new booth number → old booth released), but Epic 7 is out of scope AND unbuilt, so no upgrade record exists to render. Reclassified Partial → Not Deliverable on 2026-06-25.</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>OrderItem.parent_order_item_id (OrderItemTree, schema:1934/1944) + cart_item_type CartItemType (booth/addon/...) can nest lines, but no upgrade-specific fields exist. Requirement line 25 cross-refs external 'Booth Upgrade' story (not in brief).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>K. Onsite contact (BLOCKED — DEP-3)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Onsite contact info</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Display onsite booth contact information (name/email/phone) for the order</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED (producer unbuilt): the OnsiteBoothContact table exists (migration 20260622120000) but ZERO code writes it — no onsiteBoothContact.create/upsert/update anywhere in 5 repos. Schema doc-comment names the producer as the unbuilt 'Exhibitor Onboarding → Onsite Booth Contacts' step (later synced to HubSpot/order). The per-show display decision stands, but there is no produced data to show until that step ships → Blocked (was Deliverable; reopens DEP-3 on producer grounds).
+— prior note —
+RESOLVED (decision 2026-06-25): show ONE onsite contact PER SHOW, sourced from OnsiteBoothContact via Order.company_id + (OrderItem.show_product_id → ShowProduct → Shows).show_id. No order-level link needed; the conflicting order-level framing from epics 16/22 is out of scope and disregarded. Shows with no contact yet render a placeholder.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>13.3 mandates displaying onsite contact and defers the contract to 'View Onsite Booth Contact' (16.1/22.4/22.5), which assumes an order-level contact. Per project decision we follow the schema instead (per-show). Edit + HubSpot sync remain epics 16/22.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>OnsiteBoothContact (admin schema) has @@unique([company_id, show_id]) and contact_name/email/phone; no order_id FK. Order has no direct show_id (multi-show derived via OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>N. Gift-cert redemption (BLOCKED — DEP-9)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Financial Summary</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Gift Certificate line (applied gift-certificate amount), shown when applied</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED (producer unbuilt): NO giftCertificateRedeem.create/update anywhere — only admin read-reports (findMany/aggregate). GiftCertificatePurchase is also never created; only GiftCertificate definitions are written. The redemption/consumption flow that links a gift cert to an order and writes the applied amount does not exist → Blocked (new DEP-9; becomes deliverable once the redeem flow ships).</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>admin-backend-api/prisma/schema.prisma:2547 GiftCertificateRedeem with order_id (FK to Order), amount Decimal(10,2), @@unique([order_id, gift_certificate_purchase_id]); Order.giftCertificateRedeems[] relation. Sum of redeem.amount per order gives the gift-cert discount line; conditional display = redeems exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>J. Salesperson schedule (BLOCKED — DEP-4)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Payment Details</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Display payment schedule set by salesperson (installment dates + amounts + method)</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api, external-api-service, admin-backend-api</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED (producer unbuilt): this requirement is the schedule 'set by SALESPERSON'. admin-backend-api writes ZERO PaymentTransaction rows (createOrderFromCart creates none); every built installment producer is exhibitor self-service generating a SYSTEM equal-split (fixed cadence), not salesperson-authored dates/amounts/method → Blocked (DEP-4). Read-only display of the SYSTEM schedule would be deliverable, but the salesperson-origination this req names is unbuilt.
+— prior note —
+DISPLAY is deliverable from PaymentTransaction (installment_number, due_date, amount, status, stripe_payment_method_id). Salesperson ORIGINATION of a custom schedule is an ADMIN/salesperson-epic dependency (see DEP-4), not an Order History gap.</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Payment Schedule Visibility (19.5) confirms the SAME installment data drives a read-only schedule display at checkout (dates, method, amount per instalment). For Order History the display is deliverable from PaymentTransaction rows.</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>PaymentTransaction model (schema 2047-2082) has installment_number/total_installments/due_date/amount/status/stripe_payment_method_id. checkout.service.ts createOrderFromCart creates no PaymentTransaction rows (admin notes). Cart/CartItem have no schedule fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>A. Centralized billing service</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>13.2</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Order Listing Table</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Total Amount must come from the 'centralized billing service'.</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>NeedsClarification</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>No 'centralized billing service' module exists in any of the 5 repos (grep for BillingService/centralized = no hits). Order.total is a frozen SNAPSHOT computed by admin/exhibitor CartPricingService at checkout; external-api-service has zero total/subtotal/saving computation code and only persists/charges snapshots. If 'centralized billing service' means an authoritative external/separate service that must re-supply or validate the total at read time, that service does not exist and is out-of-repo/unprovided.</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Producer CONFIRMED built — Order.total is frozen at checkout by CartPricingService.recalculate() (exhibitor cart-pricing.service.ts:82) via 3 real order.create paths (cart.service.ts:1221, payments.service.ts:196, admin checkout.service.ts:246). The 'centralized billing service' IS this in-process pricing engine (not a separate microservice). Data is produced today → display the snapshot. Only residual is a BA wording question (frozen snapshot vs live recompute) → moved NeedsClarification→Partial.
+— prior note —
+No 'centralized billing service' module exists in any of the 5 repos (grep for BillingService/centralized = no hits). Order.total is a frozen SNAPSHOT computed by admin/exhibitor CartPricingService at checkout; external-api-service has zero total/subtotal/saving computation code and only persists/charges snapshots. If 'centralized billing service' means an authoritative external/separate service that must re-supply or validate the total at read time, that service does not exist and is out-of-repo/unprovided.</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>'Centralized billing/pricing service' is a SYSTEM-WIDE concept (also in Booth Upgrade &amp; Recommended Upsell). No such discrete service exists; pricing lives in cart-pricing (admin + exhibitor) as snapshots. For read-only Order History the snapshot on Order.total / Order.total_savings is the natural source. See DEP-7.</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>exhibitor cart-pricing.service.ts (admin) freezes Order.total; external-api-service Notes confirm 'NO pricing/billing calculation engine... all money fields arrive as frozen SNAPSHOTS'. No shared billing service module anywhere.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>A. Centralized billing service</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>E. Per-installment Overdue</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Order Listing Table</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Each payment plan has its own status Paid / Unpaid / Overdue; Overdue reflected as not fully paid (per-installment Overdue derivation).</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api, admin-backend-api, background-worker-service</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>PaymentTransaction (the de-facto payment-plan/installment model) has status enum scheduled|processing|succeeded|failed|canceled|refunded with NO 'overdue' value, and OrderStatus has no overdue either. 'Overdue' must be DERIVED (status in scheduled/failed AND due_date&lt;now) OR a new enum value added via admin-backend-api migration (background-worker-service could host an overdue-marking cron using the cart-maintenance.expireCarts template). Per-installment Paid/Unpaid is readable (succeeded vs scheduled); Overdue is not a stored state. Note 13.2 references multiple payment plans per order, but the model is a flat set of PaymentTransaction rows with no PaymentPlan grouping entity.</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>PaymentTransactionStatus enum (schema:488) has no overdue; PaymentTransaction.due_date + status present. background-worker-service has charge crons reading status='scheduled' AND due_date&lt;=now but no overdue-marking job. No PaymentPlan parent entity — installments are flat (Order.payment_mode/installments_count + N PaymentTransaction rows).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>G. Order→Show link</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Order Listing Table</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Multi-show orders shown GROUPED (not disconnected rows).</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>No denormalized show grouping exists on Order; grouping must be COMPUTED by joining OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows and aggregating per order. Data is reachable but there is no grouping read logic, and 'GROUPED' display rules (one row per order with shows listed, vs grouped-by-show) are an aggregation to build, not a stored relation.</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>One cart/order can span multiple shows via multiple OrderItem.show_product_id values, but there is no Order-&gt;Shows relation or pre-computed grouping; aggregation logic is net-new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>I. Pay-early endpoint (Partial; salesperson-set framing → DEP-4)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Order Listing Table</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Action: Pay (EARLY payment — pay before salesperson schedule; redirect to payment summary + salesperson-set payment method + card). Available only when NOT Paid in Full.</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api, external-api-service</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (INDEPENDENT single-item audit): moved Blocked→Partial. The early-pay action rests on ALREADY-PRODUCED primitives — scheduled PaymentTransaction rows carry a saved card (stripe_payment_method_id) + due_date, produced by exhibitor split checkout (payments.service.ts:261-284); the off-session charge primitive (the same one the daily cron calls), webhook reconciliation, and paid-in-full gating (Order.paid_amount/paid_in_full_at, schema:1565-66) all exist. A net-new 'pay next scheduled installment now' endpoint is buildable on these TODAY → Partial. ⚑ BA FLAG: the spec's 'salesperson-set payment method' does NOT exist (the card is the exhibitor's own) and the schedule is system-generated (fixed 30-day cadence via INSTALLMENT_INTERVAL_DAYS), not salesperson-authored — that salesperson-origination model is the separate Blocked item #56/DEP-4. On the literal salesperson-driven reading this tips to Blocked/NeedsClarification; on the as-built exhibitor self-service reading it is Partial.
+— earlier re-audit note —
+⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED — twin of #13 (the re-audit agent hit a tool error here; verdict assigned by analogy with adversarially-confirmed #13). Same blockers: no salesperson-set payment method/schedule producer + no pay-existing-order endpoint.
+— prior note —
+Charge primitives exist (external-api-service stripe.service.createPaymentIntent + saved PaymentMethod brand/last4 + PaymentTransaction.source=manual_retry) but NO endpoint to pay an existing order's outstanding/scheduled installment EARLY. exhibitor-backend-api payments module exposes only POST /payments/checkout (creates a NEW order); there is no 'pay scheduled installment ahead of schedule' route. Depends on external stories Payment Schedule Visibility and Credit Card Payment Workflow (unprovided). The 'NOT Paid in Full' gating reuses the same payment-status derivation gap (no unpaid/paid-in-full enum literal).</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Credit Card Payment Workflow (19.7) is CHECKOUT-time payment and does NOT define paying a future installment early from Order History. Early-pay is described ONLY in 13.2 -&gt; still needs a new endpoint.</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>external-api-service Notes confirm no dedicated early-pay endpoint; exhibitor payments.controller only /checkout. Building blocks (createPaymentIntent, PaymentMethod, scheduled PaymentTransaction rows) present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>E. Per-installment Overdue</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Per-plan status: Overdue</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Each payment plan / installment can be in an Overdue status (and Overdue is reflected as not fully paid).</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api, admin-backend-api, background-worker-service</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: 'Overdue' is NOT a produced status — no overdue enum and no write-path sets one; a past-due installment stays status=scheduled and the daily cron will actually attempt to charge it (scheduled→processing→succeeded/failed), so overdue is a transient/derived state with real lifecycle caveats, not a stored value. Derivable but caveated → Partial.
+— prior note —
+DELIVERABLE (re-audit 2026-06-25, adversarially confirmed, high confidence): all inputs exist and are actively produced — each installment is a real PaymentTransaction row with a populated due_date + status, written by checkout, the daily charge cron, and Stripe webhooks. 'Overdue' = status NOT IN (succeeded,refunded,canceled) AND due_date &lt; now() — a mechanical read-time derivation over the existing @@index([status,due_date]). The missing 'overdue' enum literal is a presentation convenience, not a data gap; no upstream feature is needed. (Was Partial.)</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Re-audited Partial→Deliverable. Opposite of the Booth-Upgrade failure mode: data is fully present and live. Inputs: PaymentTransaction.due_date/status (admin schema:2055/2060) + @@index([status,due_date]):2077; rows created in payments.service.ts (split loop) + checkout.service.ts; consumed by worker payment-charge cron.</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Enum at schema.prisma:488-497 lacks 'overdue'; grep 'overdue' across worker src finds only lead-distribution doc comments; PaymentTransaction.due_date (schema:2060) + @@index([status,due_date]) (2077) provide the derivation inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>I. Pay-early endpoint (Partial; salesperson-set framing → DEP-4)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Order Listing Actions</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Pay action: EARLY payment — exhibitor pays before the salesperson's schedule; redirect to a payment summary using the salesperson-set payment method + a credit/debit card.</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api, external-api-service</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25: revised Blocked→Partial to match its independently-verified twin #10. The batch audit's Blocked call over-weighted the 'salesperson-set method/schedule' wording; the early-pay capability itself is buildable on produced primitives (scheduled PaymentTransaction + saved card + off-session charge + webhook + paid-in-full fields). The pure salesperson-origination dependency remains Blocked as #56 (DEP-4). ⚑ BA flag retained on the 'salesperson-set payment method' wording.
+— earlier re-audit note —
+⟳ RE-AUDIT 2026-06-25 (built-write-path lens): BLOCKED (producer unbuilt): both premises depend on unbuilt upstream features. (1) No salesperson-set schedule/method — every PaymentTransaction producer generates a SYSTEM equal-split with fixed 30-day cadence (payments.service.ts:261/276; INSTALLMENT_INTERVAL_DAYS=30); admin/staff checkout writes NO PaymentTransaction rows. (2) No early-pay endpoint — only POST /payments/checkout exists. Becomes Deliverable once salesperson scheduling (DEP-4) + a pay-existing-order endpoint ship.
+— prior note —
+No endpoint to pay an EXISTING order's outstanding/future scheduled installment. exhibitor-backend-api payments controller exposes ONLY POST /payments/checkout (src/payments/controllers/payments.controller.ts:50) — a cart-&gt;order creation flow, not pay-an-existing-order. external-api-service has charge primitives (stripe.service.createPaymentIntent, saved PaymentMethod brand/last4, PaymentTransaction.source=manual_retry) but NO dedicated early-pay/pay-now controller route. A new 'pay order' endpoint must be built that selects scheduled PaymentTransaction rows (status=scheduled, future due_date), charges them off-schedule via the salesperson-set stripe_payment_method_id + a card, and reconciles paid_amount via the existing external-api webhook. Depends on external stories Payment Schedule Visibility + Credit Card Payment Workflow which define the redirect/payment-summary UX and which card/method is authoritative.</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Credit Card Payment Workflow (19.7) is CHECKOUT-time payment and does NOT define paying a future installment early from Order History. Early-pay is described ONLY in 13.2 -&gt; still needs a new endpoint.</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Only route is POST /payments/checkout (payments.controller.ts:50, single @Post). PaymentTransaction installment model present (schema.prisma:2045: installment_number, due_date, status, stripe_payment_method_id, source). PaymentMethod brand/last4 present (schema.prisma:963). external-api-service stripe.service.createPaymentIntent present; no early-pay route in its controllers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>G. Order→Show link</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>13.3</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Order Details Header</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Header: Event Name</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>No direct Order-&gt;Shows relation. Event Name (Shows.title) is only reachable for product/booth orders via OrderItem.show_product_id -&gt; ShowProduct.show_id -&gt; Shows. Subscription/ppl_addon order types have NO show linkage, so they have no Event Name. Multi-show orders yield multiple titles; the header implies a single event, so grouping/selection logic must be built. No new persistence needed, but a join+derivation path is required and degenerate cases (no show, multiple shows) are unhandled today.</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Shows.title (admin schema line ~2362) reached only via OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows (exhibitor schema:2625/2358). Order has no show_id. OrderItem has show_product_id Int? (schema:1919) nullable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>G. Order→Show link</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Order Details Header</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Header: City</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>City is derived through OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows.city_id -&gt; City. Same constraint as Event Name: no direct Order-&gt;City link, absent for non-show order types, and multi-city for multi-show orders. Join+derivation logic must be built; no schema gap.</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Shows.city_id Int? -&gt; City relation (admin schema:2363 / city relation). Reachable only via the OrderItem-&gt;ShowProduct-&gt;Shows path. City is nullable on Shows (city_id Int?).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>G. Order→Show link</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Order Details Header</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Header: Event Dates</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Event Dates derived from Shows.date / start_time / end_time / timezone via the OrderItem-&gt;ShowProduct-&gt;Shows path. Fields are all nullable (date DateTime?, start_time/end_time Time?, date_to_be_added TBA flag exists), so dates may be 'To Be Announced'. No direct Order-&gt;Shows relation; derivation + null/TBA handling must be built. No schema gap.</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Shows.date (Date, nullable), start_time/end_time (Time, nullable), timezone (VarChar 50), date_to_be_added Boolean TBA flag (admin schema lines ~2373-2395). Reached only via OrderItem.show_product_id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>L. Line-item type discriminator</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>OrderItem typing distinguishes booth vs add-on vs sponsorship</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>OrderItem records carry a type discriminator that separates booth, add-on, and sponsorship lines so the details page can render distinct sections with qty + unit price</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: the booth/add-on/sponsorship discriminator is the NULLABLE OrderItem.cart_item_type, produced by only ONE of four order-creating paths — the exhibitor self-service cart checkout (cart.helpers.ts:52). Admin/staff checkout, the installment-payments path, and PPL paths leave it null, so those orders cannot be sectioned. Buildable for cart-origin product orders only → Partial.
+— prior note —
+Minor: cart_item_type is nullable (CartItemType?). For cart-originated booth/add-on/sponsorship product orders (the scope of 13.3) it is populated from the cart line, but subscription/ppl_addon orders leave it null. The read service must treat null as 'not a sectioned product line', which is correct for those order types. No data-model gap for the in-scope sections.</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>OrderItem.cart_item_type=CartItemType (schema.prisma:1936) with values booth | workshop_pavilion | sponsorship | addon | booth_setup_fee | booth_cleaning_fee (schema.prisma:2728-2737) cleanly separates the three sections plus fee lines. item_type (OrderItemType product|subscription|ppl_addon) is a coarser orthogonal discriminator; cart_item_type is the one that drives the 13.3 booth/add-on/sponsorship breakdown. quantity + unit_price + amount present on every line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>M. Coupon/fee producer coverage</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Financial Summary</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Total Saving Made = actual price vs sales price, COMPUTED BY centralized billing service</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Discount / Coupon Code line (amount and applied code), shown when applied</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>The savings VALUE exists as a frozen snapshot (Order.total_savings, schema:1571 = sum of (actual - sales) deltas captured at order creation by admin CartPricingService). But there is NO 'centralized billing service' module in any of the 5 repos: billing math is split between cart-pricing (admin-backend-api) and payment/invoice handling (external-api-service). external-api-service explicitly has zero total/saving computation code (all are upstream snapshots). If the requirement mandates a single authoritative centralized billing service to (re)compute Total Saving Made, that service does not exist; if displaying the stored Order.total_savings (with per-line backing via InvoiceLineItem.original_price vs unit_price / ShowProduct.actual_price vs sales_price) suffices, it is Deliverable.</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>'Centralized billing/pricing service' is a SYSTEM-WIDE concept (also in Booth Upgrade &amp; Recommended Upsell). No such discrete service exists; pricing lives in cart-pricing (admin + exhibitor) as snapshots. For read-only Order History the snapshot on Order.total / Order.total_savings is the natural source. See DEP-7.</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>admin-backend-api/prisma/schema.prisma:1571 Order.total_savings Decimal default 0; per-line backing: InvoiceLineItem.original_price (schema:1988-2008), ShowProduct.actual_price vs sales_price, ProductBoothSizePrice/BoothSizeBasedShowProductPrices actual_price vs sales_price. No pricingService/computeTotal found in external-api-service (grep none).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>B. Booth Number</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: on the exhibitor side neither built path produces BOTH coupon fields together — the product-cart path writes coupon_amount but never coupon_code (so 'applied code' is null when a discount applied), and the PPL/addon path writes coupon_code but hardcodes coupon_amount=0 (Phase-2 TODO). Only admin checkout writes both. Coupon line degrades on exhibitor self-serve orders → Partial.
+— prior note —
+Coupon-to-order link is a snapshot only (Order.coupon_code + Order.coupon_amount); the CouponOrders join table is commented out (schema ~1752-1768). Sufficient for displaying the applied code + discount amount; no normalized relation to the CouponCode definition for richer detail.</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>admin-backend-api/prisma/schema.prisma:1540 Order.coupon_code VarChar(100); :1541 Order.coupon_amount Decimal(10,2) default 0. Conditional display drivable by coupon_amount&gt;0 / coupon_code != null.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>M. Coupon/fee producer coverage</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>13.3</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Booth/Workshop Pavilion section</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Booth Number</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>NotDeliverable</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>admin-backend-api, exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>No booth_number / boothNumber field exists anywhere in schema or code (grep over both prisma schemas and src returned no matches). OrderItem has NO metadata column (only description VarChar(255)); the free-form JsonB 'metadata' (booth size/show title) exists ONLY on CartItem, and is NOT carried onto OrderItem at checkout. So there is no stored or derivable source for a per-order assigned Booth Number. Requires a new column (migration owned by admin-backend-api; exhibitor repo uses db push) and a write path to populate it, or an external assignment source. SOURCE now identified (Social Tables booth identifier selected at booth selection/upgrade), but it is still NOT persisted on Order/OrderItem — a column + write path from the booth-selection flow is required.</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Booth Upgrade story 7.2 step 4: 'the Exhibitor shall select a booth number'; Social Tables provides booth identifiers (Booth ID/Size/Location). So Booth Number = the Social Tables booth ID chosen at booth selection/upgrade.</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>grep booth_number/boothNumber = 0 hits across admin-backend-api/prisma/schema.prisma + exhibitor-backend-api/prisma/schema.prisma + src. OrderItem model (admin schema:1919-1950) has no metadata/booth_number field; only CartItem.metadata JsonB (schema:2819) snapshots 'booth size, show title'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>C. Booth Size / Type</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Financial Summary</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Conditional display of summary lines (discount/coupon/gift cert, cleaning fee, setup fee only when applicable)</t>
+        </is>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: mixed producer coverage. Coupon line produced by all paths; setup/cleaning fees produced only by product-cart + admin checkout (NOT the installment-payments or PPL paths); the gift-cert line has NO producer at all (see #46). Conditional display is buildable for product-cart orders but degenerate for others → Partial.</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>All conditional drivers are non-null/quantitative fields: Order.coupon_amount&gt;0 / coupon_code!=null, GiftCertificateRedeem rows exist, Order.cleaning_fees&gt;0, Order.setup_fees&gt;0. Pure presentation/aggregation logic in the new order-history detail service; no data-model gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>M. Coupon/fee producer coverage</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>13.3</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Booth/Workshop Pavilion section</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Booth Size (e.g. 10x10)</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Financial Summary</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Each fee/field has backing data verified</t>
+        </is>
+      </c>
+      <c r="F20" s="20" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>No booth-size field on OrderItem; size is derivable from Product.length/width (Decimal) via OrderItem.product_id -&gt; Product, since the booth is modeled as a Product. This is a snapshot risk: OrderItem.description is the only frozen name snapshot; length/width are read live off the current Product, so if the product is later edited the displayed size may drift from purchase time. Derivation/formatting (length x width) must be built; consider snapshotting at checkout.</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Product.length / Product.width Decimal? (admin schema:1221-1222). OrderItem.product relation exists (schema:1944). OrderItem itself has no size column — only description VarChar(255).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>C. Booth Size / Type</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Booth/Workshop Pavilion section</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Booth Type (Standard/Premium/Corner)</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>No first-class Booth Type on the order line. ProductType hierarchy (ProductType.name/code, parent_type_id) classifies products as booth/sponsor/etc., but there is no confirmed Standard/Premium/Corner taxonomy in the schema/seed (no such ProductType codes found). Booth Type would be derived from OrderItem.product -&gt; Product.product_type_id -&gt; ProductType, but the exact Standard/Premium/Corner values are not modeled/seeded today, so the mapping is unproven. Same live-vs-snapshot drift risk as Booth Size.</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>ProductType model (name VarChar(100), code unique, parent_type_id hierarchy) admin schema; no Standard/Premium/Corner codes found in schema/seed. Reached via OrderItem.product_id -&gt; Product.product_type_id -&gt; ProductType. No booth_type column on OrderItem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>D. Booth Upgrade details</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Booth/Workshop Pavilion section</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Upgrade details (if any)</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api, admin-backend-api</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Data contract now known, but no dedicated upgrade fields in schema. Upgrade likely = a price-difference OrderItem (parent_order_item_id tree / cart_item_type) + capture of from-size/to-size + new booth number. Needs storage design + write path; no from/to-size or upgrade-delta column exists today.</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>RESOLVED by Booth Upgrade story (Epic 7.1/7.2). Upgrade = pick larger size -&gt; pay PRICE DIFFERENCE (computed by 'centralized pricing service') -&gt; select new booth number -&gt; old booth released. 'Upgrade details' to render = from-size -&gt; to-size, upgrade amount, new booth number.</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>OrderItem.parent_order_item_id (OrderItemTree, schema:1934/1944) + cart_item_type CartItemType (booth/addon/...) can nest lines, but no upgrade-specific fields exist. Requirement line 25 cross-refs external 'Booth Upgrade' story (not in brief).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>E. Per-installment Overdue</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Order Listing Table</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Each payment plan has its own status Paid / Unpaid / Overdue; Overdue reflected as not fully paid (per-installment Overdue derivation).</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api, admin-backend-api, background-worker-service</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>PaymentTransaction (the de-facto payment-plan/installment model) has status enum scheduled|processing|succeeded|failed|canceled|refunded with NO 'overdue' value, and OrderStatus has no overdue either. 'Overdue' must be DERIVED (status in scheduled/failed AND due_date&lt;now) OR a new enum value added via admin-backend-api migration (background-worker-service could host an overdue-marking cron using the cart-maintenance.expireCarts template). Per-installment Paid/Unpaid is readable (succeeded vs scheduled); Overdue is not a stored state. Note 13.2 references multiple payment plans per order, but the model is a flat set of PaymentTransaction rows with no PaymentPlan grouping entity.</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>PaymentTransactionStatus enum (schema:488) has no overdue; PaymentTransaction.due_date + status present. background-worker-service has charge crons reading status='scheduled' AND due_date&lt;=now but no overdue-marking job. No PaymentPlan parent entity — installments are flat (Order.payment_mode/installments_count + N PaymentTransaction rows).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>E. Per-installment Overdue</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Per-plan status: Overdue</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Each payment plan / installment can be in an Overdue status (and Overdue is reflected as not fully paid).</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api, admin-backend-api, background-worker-service</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>PaymentTransactionStatus enum (admin-backend-api/prisma/schema.prisma:488) has NO 'overdue' value (scheduled|processing|succeeded|failed|canceled|refunded). 'Overdue' is not a stored state. Two paths: (a) DERIVE at read time = status in (scheduled,failed) AND due_date &lt; now() - no migration, computed in exhibitor-backend-api read service; OR (b) add an 'overdue' enum value + an overdue-marking cron. background-worker-service has the cron home (cart-maintenance.expireCarts is the template) and reads @@index([status,due_date]) already, but enum/migration must be added in admin-backend-api (migration source of truth). If only derive-at-read is needed, this is Deliverable; the Partial reflects that no stored Overdue state exists today.</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Enum at schema.prisma:488-497 lacks 'overdue'; grep 'overdue' across worker src finds only lead-distribution doc comments; PaymentTransaction.due_date (schema:2060) + @@index([status,due_date]) (2077) provide the derivation inputs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>F. Order Payment Status</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Order Listing Table</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Column: Payment Status — order-level status derived from associated payment plan / installment statuses (Paid in Full / Partially Paid / Unpaid).</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>OrderStatus enum (schema:418) has only pending|partially_paid|completed|failed|refunded|canceled — NO literal 'unpaid' or 'paid in full'. Raw inputs exist (Order.paid_amount, paid_in_full_at, partially_paid; PaymentTransaction.status per installment) but the Paid in Full / Partially Paid / Unpaid mapping must be DERIVED in a new service (compare paid_amount vs total, roll up PaymentTransaction rows). No read-side derivation logic exists in exhibitor-backend-api.</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>OrderStatus enum lacks unpaid/paid-in-full; Order.paid_amount + paid_in_full_at + PaymentTransaction.status present (schema:488). Derivation owned on WRITE side by external-api-service webhook computeNewOrderStatus(); no exhibitor-facing read endpoint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>F. Order Payment Status</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Order Listing Table</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Action: Pay (EARLY payment — pay before salesperson schedule; redirect to payment summary + salesperson-set payment method + card). Available only when NOT Paid in Full.</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api, external-api-service</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Charge primitives exist (external-api-service stripe.service.createPaymentIntent + saved PaymentMethod brand/last4 + PaymentTransaction.source=manual_retry) but NO endpoint to pay an existing order's outstanding/scheduled installment EARLY. exhibitor-backend-api payments module exposes only POST /payments/checkout (creates a NEW order); there is no 'pay scheduled installment ahead of schedule' route. Depends on external stories Payment Schedule Visibility and Credit Card Payment Workflow (unprovided). The 'NOT Paid in Full' gating reuses the same payment-status derivation gap (no unpaid/paid-in-full enum literal).</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Credit Card Payment Workflow (19.7) is CHECKOUT-time payment and does NOT define paying a future installment early from Order History. Early-pay is described ONLY in 13.2 -&gt; still needs a new endpoint.</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>external-api-service Notes confirm no dedicated early-pay endpoint; exhibitor payments.controller only /checkout. Building blocks (createPaymentIntent, PaymentMethod, scheduled PaymentTransaction rows) present.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>F. Order Payment Status</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Order Details Header</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Header: Payment Status</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>OrderStatus enum has pending|partially_paid|completed|failed|refunded|canceled but NO literal 'unpaid'/'overdue' value. The required Paid-in-Full / Partially Paid / Unpaid (and Overdue reflected as not-fully-paid) must be DERIVED in code from Order.paid_amount vs Order.total + Order.paid_in_full_at and per-installment PaymentTransaction.status/due_date (overdue = status in scheduled/failed AND due_date&lt;now). Raw data is fully present; derivation service is unbuilt in the read repo.</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>Order.status (OrderStatus, schema:1532 region), paid_amount, paid_in_full_at; PaymentTransaction.status (scheduled|processing|succeeded|failed|canceled|refunded — no 'overdue') + due_date (schema:2045). computeNewOrderStatus() exists on the WRITE side in external-api-service webhook.service.ts, but no exhibitor-facing read derivation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>G. Order-&gt;Show link</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Order Listing Table</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Column: Associated Shows (multi-city / multi-show) per order.</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Order has NO direct show_id (verified at schema.prisma:1532-1596 — no show_id/show relation). Associated Shows is derivable ONLY via OrderItem.show_product_id (schema:1931) -&gt; ShowProduct.show_id (schema:2627) -&gt; Shows. Grouping/join logic must be built. Subscription/ppl_addon order_types have no show_product_id and therefore no associated shows.</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>No Order.show_id; OrderItem.show_product_id is nullable and only set for cart-originated product orders. ShowProduct.show_id -&gt; Shows path confirmed. Shows model carries title/city_id for the multi-city display.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>G. Order-&gt;Show link</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Order Listing Table</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Multi-show orders shown GROUPED (not disconnected rows).</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>No denormalized show grouping exists on Order; grouping must be COMPUTED by joining OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows and aggregating per order. Data is reachable but there is no grouping read logic, and 'GROUPED' display rules (one row per order with shows listed, vs grouped-by-show) are an aggregation to build, not a stored relation.</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>One cart/order can span multiple shows via multiple OrderItem.show_product_id values, but there is no Order-&gt;Shows relation or pre-computed grouping; aggregation logic is net-new.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>G. Order-&gt;Show link</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Order Details Header</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Header: Event Name</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>No direct Order-&gt;Shows relation. Event Name (Shows.title) is only reachable for product/booth orders via OrderItem.show_product_id -&gt; ShowProduct.show_id -&gt; Shows. Subscription/ppl_addon order types have NO show linkage, so they have no Event Name. Multi-show orders yield multiple titles; the header implies a single event, so grouping/selection logic must be built. No new persistence needed, but a join+derivation path is required and degenerate cases (no show, multiple shows) are unhandled today.</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Shows.title (admin schema line ~2362) reached only via OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows (exhibitor schema:2625/2358). Order has no show_id. OrderItem has show_product_id Int? (schema:1919) nullable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>G. Order-&gt;Show link</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Order Details Header</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Header: City</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>City is derived through OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows.city_id -&gt; City. Same constraint as Event Name: no direct Order-&gt;City link, absent for non-show order types, and multi-city for multi-show orders. Join+derivation logic must be built; no schema gap.</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr"/>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>Shows.city_id Int? -&gt; City relation (admin schema:2363 / city relation). Reachable only via the OrderItem-&gt;ShowProduct-&gt;Shows path. City is nullable on Shows (city_id Int?).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>G. Order-&gt;Show link</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Order Details Header</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Header: Event Dates</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>Event Dates derived from Shows.date / start_time / end_time / timezone via the OrderItem-&gt;ShowProduct-&gt;Shows path. Fields are all nullable (date DateTime?, start_time/end_time Time?, date_to_be_added TBA flag exists), so dates may be 'To Be Announced'. No direct Order-&gt;Shows relation; derivation + null/TBA handling must be built. No schema gap.</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Shows.date (Date, nullable), start_time/end_time (Time, nullable), timezone (VarChar 50), date_to_be_added Boolean TBA flag (admin schema lines ~2373-2395). Reached only via OrderItem.show_product_id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>H. Invoice PDF</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Order Listing Table</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Action: Invoice (download/view invoice PDF).</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>Invoice/InvoiceLineItem data models exist (schema:1953/1987) but Invoice has NO file_url/PDF field and no stored invoice document. A working pdfkit renderer exists but is PPL-specific (exhibitor-backend-api/src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf + S3). A product/booth order invoice PDF renderer must be generalized/built; no invoice-PDF route exists for order-history.</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>Invoice model has no PDF/file field; only PPL pdfkit renderer present in src/ppl/services/ppl.service.ts. admin-backend-api and external-api-service have no invoice PDF generation either.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>H. Invoice PDF</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Order Listing Actions</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Invoice action: download/view the order Invoice as a PDF.</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>No order-invoice PDF generator and no stored invoice file. Invoice model has NO file_url/PDF field (exhibitor-backend-api prisma/schema.prisma:1953; only file_url at line 348 is the Agreement TEMPLATE). A working pdfkit renderer exists but is PPL-specific (src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf, line 985/753) and would need generalization to product/booth orders from Invoice + InvoiceLineItem. No invoice-PDF route or service for orders exists in any repo (external-api-service and background-worker-service both lack PDF tooling).</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Invoice + InvoiceLineItem data present (schema.prisma:1953/1987) with InvoiceItemType breakdown + original_price vs unit_price; pdfkit renderer src/ppl/services/ppl.service.ts:985 reusable but PPL-scoped; no Invoice.file_url field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>H. Invoice PDF</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Payment Details</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Download invoice (per-order / per-payment invoice document)</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>Invoice/InvoiceLineItem data rows exist (with InvoiceItemType covering booth/addon/sponsorship/fees and original_price vs unit_price for savings), but Invoice has NO file_url/PDF storage field and there is no order/booth invoice PDF renderer. A working pdfkit renderer exists at exhibitor-backend-api src/ppl/services/ppl.service.ts renderInvoicePdf/downloadInvoicePdf with S3 upload, but it is PPL-invoice-specific and would need to be generalized to product/booth orders. Missing: a generalized order-invoice PDF renderer + download endpoint (no schema change strictly required since generation can be on-demand).</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>Invoice + InvoiceLineItem models present in all backends (admin schema 1953-2008); ppl.service.ts:753 downloadInvoicePdf + :985 renderInvoicePdf use pdfkit + UploadService (S3). No file_url on Invoice; no order-history invoice route.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>I. Pay-early endpoint</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Order Listing Actions</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Pay action: EARLY payment — exhibitor pays before the salesperson's schedule; redirect to a payment summary using the salesperson-set payment method + a credit/debit card.</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api, external-api-service</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>No endpoint to pay an EXISTING order's outstanding/future scheduled installment. exhibitor-backend-api payments controller exposes ONLY POST /payments/checkout (src/payments/controllers/payments.controller.ts:50) — a cart-&gt;order creation flow, not pay-an-existing-order. external-api-service has charge primitives (stripe.service.createPaymentIntent, saved PaymentMethod brand/last4, PaymentTransaction.source=manual_retry) but NO dedicated early-pay/pay-now controller route. A new 'pay order' endpoint must be built that selects scheduled PaymentTransaction rows (status=scheduled, future due_date), charges them off-schedule via the salesperson-set stripe_payment_method_id + a card, and reconciles paid_amount via the existing external-api webhook. Depends on external stories Payment Schedule Visibility + Credit Card Payment Workflow which define the redirect/payment-summary UX and which card/method is authoritative.</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>Credit Card Payment Workflow (19.7) is CHECKOUT-time payment and does NOT define paying a future installment early from Order History. Early-pay is described ONLY in 13.2 -&gt; still needs a new endpoint.</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>Only route is POST /payments/checkout (payments.controller.ts:50, single @Post). PaymentTransaction installment model present (schema.prisma:2045: installment_number, due_date, status, stripe_payment_method_id, source). PaymentMethod brand/last4 present (schema.prisma:963). external-api-service stripe.service.createPaymentIntent present; no early-pay route in its controllers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>K. Onsite contact</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Onsite contact info</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Display onsite booth contact information (name/email/phone) for the order</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>exhibitor-backend-api</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>CONFIRMED gap: stories want an order-level onsite contact, but OnsiteBoothContact is keyed (company_id, show_id) with NO order linkage. Resolve multi-show (one order spanning shows -&gt; multiple per-show contacts). Display-only for this epic.</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>View Onsite Booth Contact (16.1) + Onsite Contacts Management (22.4) + HubSpot Sync (22.5) explicitly place the onsite contact AT THE ORDER LEVEL. Order History only DISPLAYS it (View); Edit/HubSpot sync are separate epics (see DEP-3).</t>
-        </is>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>OnsiteBoothContact (admin schema) has @@unique([company_id, show_id]) and contact_name/email/phone; no order_id FK. Order has no direct show_id (multi-show derived via OrderItem.show_product_id -&gt; ShowProduct -&gt; Shows).</t>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>exhibitor-backend-api</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>⟳ RE-AUDIT 2026-06-25 (built-write-path lens): Demoted Deliverable→Partial: most fields have real producers, but two fail 'each fee/field has backing data' — TAX is hardcoded to 0 in both order producers (cart-pricing.service.ts:173, payments.service.ts:525 — Phase-2 TODO) and the gift-cert field has no producer (#46). Not every fee/field is genuinely backed by produced data → Partial.</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Every Financial Summary field has a concrete backing column on Order or a related model: subtotal (Order.subtotal:1539), coupon (Order.coupon_code:1540/coupon_amount:1541), gift cert (GiftCertificateRedeem.amount:2553), cleaning fee (Order.cleaning_fees:1570), setup fee (Order.setup_fees:1569), total savings (Order.total_savings:1571), total paid (Order.paid_amount:1565), total (Order.total:1543). All verified present in admin-backend-api/prisma/schema.prisma (shared DB).</t>
         </is>
       </c>
     </row>
@@ -4465,7 +4498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4475,6 +4508,7 @@
     <col width="78" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4513,6 +4547,11 @@
           <t>Why it matters / what it blocks</t>
         </is>
       </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Status / Resolution</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
@@ -4548,6 +4587,11 @@
           <t>Affects 13.2 Total Amount, 13.3 Financial Summary / Total Saving</t>
         </is>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Open (narrowed 2026-06-25). Producer CONFIRMED built — Order.total is frozen at checkout by CartPricingService.recalculate(); the data is displayable from the snapshot TODAY. The 'centralized billing service' is that in-process engine, not a separate service. Residual is purely the wording/architecture question (show frozen snapshot vs call a live recompute). Verdict moved NeedsClarification→Partial.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
@@ -4583,6 +4627,11 @@
           <t>Blocks 13.3 Onsite contact display (DEP-3)</t>
         </is>
       </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-06-25 — Decision: disregard the out-of-scope epics' (16/22) order-level framing; follow the DB schema and show ONE onsite contact PER SHOW (grouped under each booked show). 13.3 mandates the display; it defers the data contract to 'View Onsite Booth Contact', whose order-level assumption the (company_id, show_id) model can't satisfy — so we source per show via OrderItem.show_product_id → ShowProduct → Shows + (company_id, show_id). A booked show with no contact yet renders a 'No onsite contact added yet' placeholder.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -4618,6 +4667,11 @@
           <t>Blocks 13.2 Pay action + new early-pay endpoint design</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -4653,6 +4707,11 @@
           <t>Blocks 13.3 Booth Number (only Not-Deliverable; DEP-1)</t>
         </is>
       </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -4660,22 +4719,22 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>13.2 / 13.3</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Booth upgrade representation on the order</t>
+          <t>Overdue + payment-status labels</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Is a booth upgrade recorded as an amendment to the original Order (a new price-difference line on the same order) or as a separate order? This determines how 'Upgrade details' render in Order History and what must be stored (from/to size, upgrade amount, new booth number).</t>
+          <t>PaymentTransactionStatus has no 'overdue' value and OrderStatus has no 'unpaid'/'paid in full' literal. Should Overdue be a PERSISTED status (admin-backend-api enum migration + a background-worker overdue-marking cron) or derived at read time (due_date &lt; now AND not succeeded)? And confirm the exact order-level label set (Paid in Full / Partially Paid / Unpaid) and whether Overdue surfaces as a distinct badge.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -4685,7 +4744,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Affects 13.3 Booth Upgrade details (DEP-2)</t>
+          <t>Affects 13.2 + 13.3 payment status</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-06-25 — Decision: use the 3-value order-level set (Paid in Full / Partially Paid / Unpaid), computed AT RUNTIME as a DERIVED value (not stored — no DB enum/column added). Overdue is a per-plan status that rolls up into Partially Paid/Unpaid (no separate order-level badge); derive at read time (due_date &lt; now AND not succeeded). Persist-vs-derive is an implementation choice (we derive), not a BA question. ⚑ FLAG FOR BA: the 13.2 listing-row spec says 'Payment Status (Paid, Unpaid)' — a 2-value shorthand that omits 'Partially Paid' and writes 'Paid' instead of 'Paid in Full'; confirm the listing row uses the same canonical 3-value derived status as the details page (story wording cleanup). ⚠ CODE NOTE (verified 2026-06-25): OrderStatus.refunded is NEVER assigned to an Order — the charge.refunded webhook only flips PaymentTransaction→refunded and voids the Invoice; Order.status is only ever written to pending/partially_paid/completed/failed/canceled. So a refunded order keeps its prior status (usually 'completed'/Paid in Full) and refunds are INVISIBLE at the order level. If the order-level Payment Status must reflect refunds, it cannot be read from OrderStatus alone — derive from PaymentTransaction.refunded / Invoice.void. Same blind spot for both full and split mode.</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4759,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -4705,12 +4769,12 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Overdue + payment-status labels</t>
+          <t>Non-show order types in Order History</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>PaymentTransactionStatus has no 'overdue' value and OrderStatus has no 'unpaid'/'paid in full' literal. Should Overdue be a PERSISTED status (admin-backend-api enum migration + a background-worker overdue-marking cron) or derived at read time (due_date &lt; now AND not succeeded)? And confirm the exact order-level label set (Paid in Full / Partially Paid / Unpaid) and whether Overdue surfaces as a distinct badge.</t>
+          <t>Order has no direct show link; shows/city/dates are derived via OrderItem -&gt; ShowProduct -&gt; Shows. Subscription / PPL-addon orders have NO show linkage. Should those order types appear in Order History at all, and if so what do the Associated Shows / Event Name / City / Event Dates columns show?</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -4720,7 +4784,12 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Affects 13.2 + 13.3 payment status</t>
+          <t>Affects 13.2 listing + 13.3 header</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4730,32 +4799,37 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Display</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>13.2 / 13.3</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Non-show order types in Order History</t>
+          <t>Order ID + canceled/refunded orders</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Order has no direct show link; shows/city/dates are derived via OrderItem -&gt; ShowProduct -&gt; Shows. Subscription / PPL-addon orders have NO show linkage. Should those order types appear in Order History at all, and if so what do the Associated Shows / Event Name / City / Event Dates columns show?</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Should 'Order ID' display Order.order_number (e.g. ORD-2026-00001) or the numeric id? And should canceled / failed / soft-deleted (deleted_at != null) orders appear in the Order History list, and how does their Payment Status render?</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Affects 13.2 listing + 13.3 header</t>
+          <t>Affects 13.1 / 13.2 listing</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4765,32 +4839,37 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Display</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>13.2 / 13.3</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Order ID + canceled/refunded orders</t>
+          <t>Invoice PDF generation approach</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Should 'Order ID' display Order.order_number (e.g. ORD-2026-00001) or the numeric id? And should canceled / failed / soft-deleted (deleted_at != null) orders appear in the Order History list, and how does their Payment Status render?</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Invoice has no stored PDF; a pdfkit+S3 renderer exists but is PPL-specific. Should the order Invoice PDF reuse/generalize that renderer (on-demand), be pre-rendered and stored (new Invoice.file_url column + S3), or is invoice PDF owned by an external/QuickBooks flow (Order.quickbooks_order_id exists)? Is one invoice per order or per installment (PaymentTransaction.invoice_id)?</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Affects 13.1 / 13.2 listing</t>
+          <t>Affects 13.2 Invoice action + 13.3 download invoice (DEP-6)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4805,17 +4884,17 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>13.2 / 13.3</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Invoice PDF generation approach</t>
+          <t>Signed agreement document for booth/product orders</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Invoice has no stored PDF; a pdfkit+S3 renderer exists but is PPL-specific. Should the order Invoice PDF reuse/generalize that renderer (on-demand), be pre-rendered and stored (new Invoice.file_url column + S3), or is invoice PDF owned by an external/QuickBooks flow (Order.quickbooks_order_id exists)? Is one invoice per order or per installment (PaymentTransaction.invoice_id)?</t>
+          <t>OrderAgreement stores signature data + acceptance timestamp but no rendered signed-document file. For non-PPL (booth/product) orders, is a downloadable signed agreement document expected, and should it reuse the PPL signed-doc renderer?</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -4825,42 +4904,12 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Affects 13.2 Invoice action + 13.3 download invoice (DEP-6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Documents</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>13.3</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Signed agreement document for booth/product orders</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>OrderAgreement stores signature data + acceptance timestamp but no rendered signed-document file. For non-PPL (booth/product) orders, is a downloadable signed agreement document expected, and should it reuse the PPL signed-doc renderer?</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
           <t>Affects 13.3 Download signed agreement (DEP-5)</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4942,7 +4991,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>13.3 Booth Number (only Not-Deliverable item)</t>
+          <t>13.3 Booth Number (#26 — BLOCKED, was Not-Deliverable)</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
@@ -4979,7 +5028,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>13.3 Upgrade details</t>
+          <t>13.3 Upgrade details (#33 — BLOCKED, was Not-Deliverable)</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -5016,7 +5065,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>13.3 Onsite contact info display</t>
+          <t>13.3 Onsite contact info display (#36 — now BLOCKED)</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -5026,7 +5075,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>OnsiteBoothContact is keyed (company_id, show_id) with NO order linkage. The order-level association is established by Epic 22. Order History only VIEWS the contact; Edit + HubSpot sync are Epic 16/22 scope.</t>
+          <t>RE-AUDIT 2026-06-25: the per-show display DECISION stands, but OnsiteBoothContact has NO write-path anywhere in the 5 repos — its producer is the unbuilt 'Exhibitor Onboarding → Onsite Booth Contacts' step. So there is no produced data to display until that onboarding step ships. Reopened as a producer (data-production) blocker, distinct from the earlier order-level-framing question.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -5053,7 +5102,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>13.3 Display payment schedule; indirectly 13.2/13.3 payment-status derivation</t>
+          <t>13.3 Salesperson payment schedule #56 (BLOCKED). Early-pay #10/#13 is Partial — buildable on produced primitives — but its salesperson-set-method/schedule framing also depends on this.</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -5063,7 +5112,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Order History DISPLAY is deliverable from PaymentTransaction rows, but those must be ORIGINATED by the salesperson/checkout flow. Not defined in the exhibitor stories.</t>
+          <t>RE-AUDIT 2026-06-25: admin-backend-api writes ZERO PaymentTransaction rows (createOrderFromCart creates none); only exhibitor self-service produces a SYSTEM equal-split (fixed 30-day cadence). The salesperson-originated schedule (#56) is BLOCKED until this ships. The early-pay ACTION (#10/#13) is Partial: an exhibitor can pay a scheduled installment early on their own saved card today; only the literal 'salesperson-set method/schedule' wording leans on this dependency.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -5217,6 +5266,43 @@
       <c r="G9" s="5" t="inlineStr">
         <is>
           <t>external-api-service (webhook) + background-worker-service (cron)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>DEP-9</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Gift-certificate redemption flow — Checkout / Gift-cert epic</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>A built redeem/consumption path that links a purchased gift certificate to an order and writes GiftCertificateRedeem.amount</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>13.3 Gift Certificate line (#46 — BLOCKED)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Hard (blocks)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>No giftCertificateRedeem.create/update exists in any repo (only admin read-reports + GiftCertificate definitions). The Financial-Summary gift-cert line has no produced data until the redemption flow is built.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Checkout / Gift-certificate epic (admin + exhibitor)</t>
         </is>
       </c>
     </row>

</xml_diff>